<commit_message>
fix: C01 project import template 6→19 fields, C02 supplier contract import full fields
</commit_message>
<xml_diff>
--- a/backend/templates/项目导入模板.xlsx
+++ b/backend/templates/项目导入模板.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:S2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,27 +424,92 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>合同编号</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>合同类型</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>业主单位</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>联系人</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>联系电话</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>合同金额</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>预算金额</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>签订时间</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>合同开始时间</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>合同结束时间</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>所属年度</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>所属部门</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>负责人</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
         <is>
           <t>集团内外</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>项目类型</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>合同状态</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>ERP项目编号</t>
         </is>
       </c>
     </row>
@@ -456,29 +521,80 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>CT-2026-001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>框架合同</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>中国移动崇左分公司</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>张经理</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0771-1234567</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="H2" t="n">
+        <v>950000</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>2026-12-31</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="L2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>数智工程部</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>一游</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
         <is>
           <t>集团内</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>工程施工</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>执行中</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>